<commit_message>
Add stop-loss backtests, model comparison chart, sector target weights, README docs
</commit_message>
<xml_diff>
--- a/portfolio_model/outputs/spreadsheet/portfolio_analysis.xlsx
+++ b/portfolio_model/outputs/spreadsheet/portfolio_analysis.xlsx
@@ -24,6 +24,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investment Theses" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Quality" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scorecard" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stop-Loss Backtests" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -524,7 +525,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-04 18:47 UTC | Seed: 42 | Simulations: 10000 | Model version: 1.0.0</t>
+          <t>Generated: 2026-10-04 18:50 UTC | Seed: 42 | Simulations: 10000 | Model version: 1.0.0</t>
         </is>
       </c>
     </row>
@@ -4789,7 +4790,7 @@
       </c>
       <c r="D6" s="16" t="inlineStr">
         <is>
-          <t>{'status': 'ok', 'inception': '2000-01-03', 'rows': 6728, 'fetched_utc': '2026-10-04T18:47:49.055074+00:00'}</t>
+          <t>{'status': 'ok', 'inception': '2000-01-03', 'rows': 6728, 'fetched_utc': '2026-10-04T18:50:25.797519+00:00'}</t>
         </is>
       </c>
     </row>
@@ -4811,7 +4812,7 @@
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>{'status': 'ok', 'inception': '2000-01-03', 'rows': 6728, 'fetched_utc': '2026-10-04T18:47:49.057353+00:00'}</t>
+          <t>{'status': 'ok', 'inception': '2000-01-03', 'rows': 6728, 'fetched_utc': '2026-10-04T18:50:25.800034+00:00'}</t>
         </is>
       </c>
     </row>
@@ -4833,7 +4834,7 @@
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t>{'status': 'ok', 'inception': '2021-07-28', 'rows': 1302, 'fetched_utc': '2026-10-04T18:47:49.059485+00:00'}</t>
+          <t>{'status': 'ok', 'inception': '2021-07-28', 'rows': 1302, 'fetched_utc': '2026-10-04T18:50:25.801697+00:00'}</t>
         </is>
       </c>
     </row>
@@ -4855,7 +4856,7 @@
       </c>
       <c r="D9" s="16" t="inlineStr">
         <is>
-          <t>{'status': 'ok', 'inception': '2002-07-30', 'rows': 6084, 'fetched_utc': '2026-10-04T18:47:49.061306+00:00'}</t>
+          <t>{'status': 'ok', 'inception': '2002-07-30', 'rows': 6084, 'fetched_utc': '2026-10-04T18:50:25.803463+00:00'}</t>
         </is>
       </c>
     </row>
@@ -4877,7 +4878,7 @@
       </c>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>{'status': 'ok', 'inception': '2002-07-30', 'rows': 6084, 'fetched_utc': '2026-10-04T18:47:49.062973+00:00'}</t>
+          <t>{'status': 'ok', 'inception': '2002-07-30', 'rows': 6084, 'fetched_utc': '2026-10-04T18:50:25.805187+00:00'}</t>
         </is>
       </c>
     </row>
@@ -4899,7 +4900,7 @@
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>{'status': 'ok', 'inception': '2010-09-09', 'rows': 4041, 'fetched_utc': '2026-10-04T18:47:49.064882+00:00'}</t>
+          <t>{'status': 'ok', 'inception': '2010-09-09', 'rows': 4041, 'fetched_utc': '2026-10-04T18:50:25.806728+00:00'}</t>
         </is>
       </c>
     </row>
@@ -4921,7 +4922,7 @@
       </c>
       <c r="D12" s="16" t="inlineStr">
         <is>
-          <t>{'status': 'ok', 'inception': '2000-01-03', 'rows': 6728, 'fetched_utc': '2026-10-04T18:47:49.067067+00:00'}</t>
+          <t>{'status': 'ok', 'inception': '2000-01-03', 'rows': 6728, 'fetched_utc': '2026-10-04T18:50:25.808489+00:00'}</t>
         </is>
       </c>
     </row>
@@ -4943,7 +4944,7 @@
       </c>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>{'status': 'ok', 'inception': '2003-09-29', 'rows': 5790, 'fetched_utc': '2026-10-04T18:47:49.068793+00:00'}</t>
+          <t>{'status': 'ok', 'inception': '2003-09-29', 'rows': 5790, 'fetched_utc': '2026-10-04T18:50:25.810154+00:00'}</t>
         </is>
       </c>
     </row>
@@ -5590,6 +5591,2516 @@
       <c r="F27" s="10" t="inlineStr">
         <is>
           <t>P1 Critical</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="23" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="42" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Stop-Loss Backtests (historical, not advice)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>ticker</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>mode</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>level</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>cagr</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>vol</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>sharpe</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>sortino</t>
+        </is>
+      </c>
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t>max_drawdown</t>
+        </is>
+      </c>
+      <c r="I3" s="9" t="inlineStr">
+        <is>
+          <t>total_return</t>
+        </is>
+      </c>
+      <c r="J3" s="9" t="inlineStr">
+        <is>
+          <t>exits</t>
+        </is>
+      </c>
+      <c r="K3" s="9" t="inlineStr">
+        <is>
+          <t>turnover</t>
+        </is>
+      </c>
+      <c r="L3" s="9" t="inlineStr">
+        <is>
+          <t>missed_upside</t>
+        </is>
+      </c>
+      <c r="M3" s="9" t="inlineStr">
+        <is>
+          <t>reentry_days</t>
+        </is>
+      </c>
+      <c r="N3" s="9" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="n">
+        <v/>
+      </c>
+      <c r="D4" s="11" t="n">
+        <v>0.1056477327058141</v>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>0.4213253873361095</v>
+      </c>
+      <c r="F4" s="10" t="n">
+        <v>0.4500467123039825</v>
+      </c>
+      <c r="G4" s="10" t="n">
+        <v>0.5948922664284093</v>
+      </c>
+      <c r="H4" s="11" t="n">
+        <v>-0.7988731794932153</v>
+      </c>
+      <c r="I4" s="11" t="n">
+        <v>13.60490660949948</v>
+      </c>
+      <c r="J4" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>0.04333410037786645</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>0.3808985868135027</v>
+      </c>
+      <c r="F5" s="10" t="n">
+        <v>0.3024574566004236</v>
+      </c>
+      <c r="G5" s="10" t="n">
+        <v>0.3927817450261595</v>
+      </c>
+      <c r="H5" s="11" t="n">
+        <v>-0.8433772282571956</v>
+      </c>
+      <c r="I5" s="11" t="n">
+        <v>2.103147965050269</v>
+      </c>
+      <c r="J5" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="K5" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="L5" s="11" t="n">
+        <v>1.987099071931526</v>
+      </c>
+      <c r="M5" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N5" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>0.07507433755581072</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>0.4060459850090875</v>
+      </c>
+      <c r="F6" s="10" t="n">
+        <v>0.3827143334361712</v>
+      </c>
+      <c r="G6" s="10" t="n">
+        <v>0.496826617070116</v>
+      </c>
+      <c r="H6" s="11" t="n">
+        <v>-0.7434811353827333</v>
+      </c>
+      <c r="I6" s="11" t="n">
+        <v>5.906104786860729</v>
+      </c>
+      <c r="J6" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="K6" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="L6" s="11" t="n">
+        <v>0.9141425530617884</v>
+      </c>
+      <c r="M6" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N6" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>0.08987815961461898</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>0.4120599366048215</v>
+      </c>
+      <c r="F7" s="10" t="n">
+        <v>0.416222139537751</v>
+      </c>
+      <c r="G7" s="10" t="n">
+        <v>0.5431011019718975</v>
+      </c>
+      <c r="H7" s="11" t="n">
+        <v>-0.8508302248275315</v>
+      </c>
+      <c r="I7" s="11" t="n">
+        <v>8.949095557881165</v>
+      </c>
+      <c r="J7" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="K7" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L7" s="11" t="n">
+        <v>0.4841257534277288</v>
+      </c>
+      <c r="M7" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N7" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>0.09873843840412477</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>0.4136080577492259</v>
+      </c>
+      <c r="F8" s="10" t="n">
+        <v>0.4345595122344825</v>
+      </c>
+      <c r="G8" s="10" t="n">
+        <v>0.583152664060407</v>
+      </c>
+      <c r="H8" s="11" t="n">
+        <v>-0.8148395028603723</v>
+      </c>
+      <c r="I8" s="11" t="n">
+        <v>11.3495492130162</v>
+      </c>
+      <c r="J8" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="L8" s="11" t="n">
+        <v>0.2644612436584381</v>
+      </c>
+      <c r="M8" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N8" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>trailing</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D9" s="11" t="n">
+        <v>0.02375507750185046</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>0.3285681149493113</v>
+      </c>
+      <c r="F9" s="10" t="n">
+        <v>0.2367262031189514</v>
+      </c>
+      <c r="G9" s="10" t="n">
+        <v>0.2806795140856809</v>
+      </c>
+      <c r="H9" s="11" t="n">
+        <v>-0.8749236366128393</v>
+      </c>
+      <c r="I9" s="11" t="n">
+        <v>0.8714506981228347</v>
+      </c>
+      <c r="J9" s="10" t="n">
+        <v>59</v>
+      </c>
+      <c r="K9" s="10" t="n">
+        <v>117</v>
+      </c>
+      <c r="L9" s="11" t="n">
+        <v>2.986136932736587</v>
+      </c>
+      <c r="M9" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N9" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>trailing</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D10" s="11" t="n">
+        <v>0.0906132753518234</v>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>0.362881437377765</v>
+      </c>
+      <c r="F10" s="10" t="n">
+        <v>0.4221323387171251</v>
+      </c>
+      <c r="G10" s="10" t="n">
+        <v>0.5189736308577927</v>
+      </c>
+      <c r="H10" s="11" t="n">
+        <v>-0.8396414812946937</v>
+      </c>
+      <c r="I10" s="11" t="n">
+        <v>9.129792235103587</v>
+      </c>
+      <c r="J10" s="10" t="n">
+        <v>37</v>
+      </c>
+      <c r="K10" s="10" t="n">
+        <v>73</v>
+      </c>
+      <c r="L10" s="11" t="n">
+        <v>0.9732875292324366</v>
+      </c>
+      <c r="M10" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N10" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>trailing</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>0.07514726813743411</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>0.383062969583496</v>
+      </c>
+      <c r="F11" s="10" t="n">
+        <v>0.3820729488129694</v>
+      </c>
+      <c r="G11" s="10" t="n">
+        <v>0.4812987284920595</v>
+      </c>
+      <c r="H11" s="11" t="n">
+        <v>-0.7989064118869299</v>
+      </c>
+      <c r="I11" s="11" t="n">
+        <v>5.918621888474384</v>
+      </c>
+      <c r="J11" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="K11" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="L11" s="11" t="n">
+        <v>1.155503579239567</v>
+      </c>
+      <c r="M11" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N11" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="n">
+        <v/>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>0.0584750624215673</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>0.3046931693429364</v>
+      </c>
+      <c r="F12" s="10" t="n">
+        <v>0.3385487158378774</v>
+      </c>
+      <c r="G12" s="10" t="n">
+        <v>0.4748947185677542</v>
+      </c>
+      <c r="H12" s="11" t="n">
+        <v>-0.6788079582129238</v>
+      </c>
+      <c r="I12" s="11" t="n">
+        <v>3.559672597467387</v>
+      </c>
+      <c r="J12" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D13" s="11" t="n">
+        <v>0.03361307782262157</v>
+      </c>
+      <c r="E13" s="11" t="n">
+        <v>0.289283888335773</v>
+      </c>
+      <c r="F13" s="10" t="n">
+        <v>0.258406345105917</v>
+      </c>
+      <c r="G13" s="10" t="n">
+        <v>0.3588992003222063</v>
+      </c>
+      <c r="H13" s="11" t="n">
+        <v>-0.7924389838970872</v>
+      </c>
+      <c r="I13" s="11" t="n">
+        <v>1.417011496667616</v>
+      </c>
+      <c r="J13" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="K13" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="L13" s="11" t="n">
+        <v>0.7585499518433978</v>
+      </c>
+      <c r="M13" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N13" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D14" s="11" t="n">
+        <v>0.06704552730367386</v>
+      </c>
+      <c r="E14" s="11" t="n">
+        <v>0.2984070864036199</v>
+      </c>
+      <c r="F14" s="10" t="n">
+        <v>0.3660472367355085</v>
+      </c>
+      <c r="G14" s="10" t="n">
+        <v>0.5223509175050569</v>
+      </c>
+      <c r="H14" s="11" t="n">
+        <v>-0.6071516370474518</v>
+      </c>
+      <c r="I14" s="11" t="n">
+        <v>4.653640453449366</v>
+      </c>
+      <c r="J14" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="K14" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="L14" s="11" t="n">
+        <v>-0.1618290350977913</v>
+      </c>
+      <c r="M14" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N14" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D15" s="11" t="n">
+        <v>0.06466956412794223</v>
+      </c>
+      <c r="E15" s="11" t="n">
+        <v>0.2994702043303814</v>
+      </c>
+      <c r="F15" s="10" t="n">
+        <v>0.3583750950650276</v>
+      </c>
+      <c r="G15" s="10" t="n">
+        <v>0.5100121262806055</v>
+      </c>
+      <c r="H15" s="11" t="n">
+        <v>-0.6146711513244307</v>
+      </c>
+      <c r="I15" s="11" t="n">
+        <v>4.327028346656062</v>
+      </c>
+      <c r="J15" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="K15" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="L15" s="11" t="n">
+        <v>-0.1108846511372912</v>
+      </c>
+      <c r="M15" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N15" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D16" s="11" t="n">
+        <v>0.05471620026182822</v>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>0.301532652712724</v>
+      </c>
+      <c r="F16" s="10" t="n">
+        <v>0.3271189803494122</v>
+      </c>
+      <c r="G16" s="10" t="n">
+        <v>0.4571455024941573</v>
+      </c>
+      <c r="H16" s="11" t="n">
+        <v>-0.7001259030666498</v>
+      </c>
+      <c r="I16" s="11" t="n">
+        <v>3.145648114026413</v>
+      </c>
+      <c r="J16" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="K16" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="L16" s="11" t="n">
+        <v>0.1209728570768318</v>
+      </c>
+      <c r="M16" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N16" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>trailing</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>0.03633515953887279</v>
+      </c>
+      <c r="E17" s="11" t="n">
+        <v>0.2564258646167044</v>
+      </c>
+      <c r="F17" s="10" t="n">
+        <v>0.2671284518245004</v>
+      </c>
+      <c r="G17" s="10" t="n">
+        <v>0.3572043943604543</v>
+      </c>
+      <c r="H17" s="11" t="n">
+        <v>-0.7697797218098348</v>
+      </c>
+      <c r="I17" s="11" t="n">
+        <v>1.592806452142319</v>
+      </c>
+      <c r="J17" s="10" t="n">
+        <v>40</v>
+      </c>
+      <c r="K17" s="10" t="n">
+        <v>80</v>
+      </c>
+      <c r="L17" s="11" t="n">
+        <v>0.9255009597798955</v>
+      </c>
+      <c r="M17" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N17" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>trailing</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D18" s="11" t="n">
+        <v>0.06719395367003167</v>
+      </c>
+      <c r="E18" s="11" t="n">
+        <v>0.2709347037476466</v>
+      </c>
+      <c r="F18" s="10" t="n">
+        <v>0.3751893958990684</v>
+      </c>
+      <c r="G18" s="10" t="n">
+        <v>0.5173636117121397</v>
+      </c>
+      <c r="H18" s="11" t="n">
+        <v>-0.6036786428646497</v>
+      </c>
+      <c r="I18" s="11" t="n">
+        <v>4.674671141465319</v>
+      </c>
+      <c r="J18" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="K18" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="L18" s="11" t="n">
+        <v>0.04049514189701764</v>
+      </c>
+      <c r="M18" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N18" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>trailing</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D19" s="11" t="n">
+        <v>0.07502464095269379</v>
+      </c>
+      <c r="E19" s="11" t="n">
+        <v>0.2792798323722112</v>
+      </c>
+      <c r="F19" s="10" t="n">
+        <v>0.3980992429200452</v>
+      </c>
+      <c r="G19" s="10" t="n">
+        <v>0.567673981276738</v>
+      </c>
+      <c r="H19" s="11" t="n">
+        <v>-0.5284632021083417</v>
+      </c>
+      <c r="I19" s="11" t="n">
+        <v>5.897587831647302</v>
+      </c>
+      <c r="J19" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="K19" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="L19" s="11" t="n">
+        <v>-0.2138832132397379</v>
+      </c>
+      <c r="M19" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N19" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>DUOL</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="n">
+        <v/>
+      </c>
+      <c r="D20" s="11" t="n">
+        <v>0.01402235087081638</v>
+      </c>
+      <c r="E20" s="11" t="n">
+        <v>0.6598708221962798</v>
+      </c>
+      <c r="F20" s="10" t="n">
+        <v>0.3480715960671825</v>
+      </c>
+      <c r="G20" s="10" t="n">
+        <v>0.5201120177468026</v>
+      </c>
+      <c r="H20" s="11" t="n">
+        <v>-0.8334874602373472</v>
+      </c>
+      <c r="I20" s="11" t="n">
+        <v>0.07459684202008288</v>
+      </c>
+      <c r="J20" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>DUOL</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D21" s="11" t="n">
+        <v>-0.1123200412694773</v>
+      </c>
+      <c r="E21" s="11" t="n">
+        <v>0.5732373697414401</v>
+      </c>
+      <c r="F21" s="10" t="n">
+        <v>0.07926922843011082</v>
+      </c>
+      <c r="G21" s="10" t="n">
+        <v>0.1055064882524025</v>
+      </c>
+      <c r="H21" s="11" t="n">
+        <v>-0.8334874602373471</v>
+      </c>
+      <c r="I21" s="11" t="n">
+        <v>-0.4594156418970015</v>
+      </c>
+      <c r="J21" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="K21" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="L21" s="11" t="n">
+        <v>0.9520983835391278</v>
+      </c>
+      <c r="M21" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N21" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>DUOL</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D22" s="11" t="n">
+        <v>-0.05725142325768773</v>
+      </c>
+      <c r="E22" s="11" t="n">
+        <v>0.5995582460666489</v>
+      </c>
+      <c r="F22" s="10" t="n">
+        <v>0.2013578356974359</v>
+      </c>
+      <c r="G22" s="10" t="n">
+        <v>0.2814045700093137</v>
+      </c>
+      <c r="H22" s="11" t="n">
+        <v>-0.8334874602373472</v>
+      </c>
+      <c r="I22" s="11" t="n">
+        <v>-0.2624122787303765</v>
+      </c>
+      <c r="J22" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="K22" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="L22" s="11" t="n">
+        <v>0.5634211910734011</v>
+      </c>
+      <c r="M22" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N22" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>DUOL</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D23" s="11" t="n">
+        <v>-0.05280324252933744</v>
+      </c>
+      <c r="E23" s="11" t="n">
+        <v>0.6227199703769176</v>
+      </c>
+      <c r="F23" s="10" t="n">
+        <v>0.2243209773360098</v>
+      </c>
+      <c r="G23" s="10" t="n">
+        <v>0.3133050406441812</v>
+      </c>
+      <c r="H23" s="11" t="n">
+        <v>-0.8334874602373473</v>
+      </c>
+      <c r="I23" s="11" t="n">
+        <v>-0.2442678960517294</v>
+      </c>
+      <c r="J23" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="K23" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="L23" s="11" t="n">
+        <v>0.4655188679450274</v>
+      </c>
+      <c r="M23" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N23" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>DUOL</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D24" s="11" t="n">
+        <v>-0.1105874380608919</v>
+      </c>
+      <c r="E24" s="11" t="n">
+        <v>0.6200293263421957</v>
+      </c>
+      <c r="F24" s="10" t="n">
+        <v>0.121178488134242</v>
+      </c>
+      <c r="G24" s="10" t="n">
+        <v>0.1706724415745379</v>
+      </c>
+      <c r="H24" s="11" t="n">
+        <v>-0.8360911185686324</v>
+      </c>
+      <c r="I24" s="11" t="n">
+        <v>-0.4539461463389128</v>
+      </c>
+      <c r="J24" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="K24" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="L24" s="11" t="n">
+        <v>0.7987965335463224</v>
+      </c>
+      <c r="M24" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N24" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>DUOL</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>trailing</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D25" s="11" t="n">
+        <v>-0.1225732534494648</v>
+      </c>
+      <c r="E25" s="11" t="n">
+        <v>0.4468406898246396</v>
+      </c>
+      <c r="F25" s="10" t="n">
+        <v>-0.07016037279672843</v>
+      </c>
+      <c r="G25" s="10" t="n">
+        <v>-0.08173094841400699</v>
+      </c>
+      <c r="H25" s="11" t="n">
+        <v>-0.7350358151692828</v>
+      </c>
+      <c r="I25" s="11" t="n">
+        <v>-0.4908862309736607</v>
+      </c>
+      <c r="J25" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="K25" s="10" t="n">
+        <v>49</v>
+      </c>
+      <c r="L25" s="11" t="n">
+        <v>1.348545058120897</v>
+      </c>
+      <c r="M25" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N25" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>DUOL</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>trailing</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D26" s="11" t="n">
+        <v>0.03557136623897805</v>
+      </c>
+      <c r="E26" s="11" t="n">
+        <v>0.5333806823089525</v>
+      </c>
+      <c r="F26" s="10" t="n">
+        <v>0.3299231930949357</v>
+      </c>
+      <c r="G26" s="10" t="n">
+        <v>0.424779061626277</v>
+      </c>
+      <c r="H26" s="11" t="n">
+        <v>-0.7576587206310881</v>
+      </c>
+      <c r="I26" s="11" t="n">
+        <v>0.1977603583195127</v>
+      </c>
+      <c r="J26" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="K26" s="10" t="n">
+        <v>32</v>
+      </c>
+      <c r="L26" s="11" t="n">
+        <v>0.2781877463947019</v>
+      </c>
+      <c r="M26" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N26" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>DUOL</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>trailing</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D27" s="11" t="n">
+        <v>-0.1234133603813098</v>
+      </c>
+      <c r="E27" s="11" t="n">
+        <v>0.5463526612123289</v>
+      </c>
+      <c r="F27" s="10" t="n">
+        <v>0.03129350459110046</v>
+      </c>
+      <c r="G27" s="10" t="n">
+        <v>0.04055110877404131</v>
+      </c>
+      <c r="H27" s="11" t="n">
+        <v>-0.7988565404433809</v>
+      </c>
+      <c r="I27" s="11" t="n">
+        <v>-0.4933978272893468</v>
+      </c>
+      <c r="J27" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="K27" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="L27" s="11" t="n">
+        <v>1.098423683688364</v>
+      </c>
+      <c r="M27" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N27" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>IEF</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="n">
+        <v/>
+      </c>
+      <c r="D28" s="11" t="n">
+        <v>0.03370417651503521</v>
+      </c>
+      <c r="E28" s="11" t="n">
+        <v>0.06789490615528326</v>
+      </c>
+      <c r="F28" s="10" t="n">
+        <v>0.5221973283652125</v>
+      </c>
+      <c r="G28" s="10" t="n">
+        <v>0.7982584381984438</v>
+      </c>
+      <c r="H28" s="11" t="n">
+        <v>-0.2392477452272798</v>
+      </c>
+      <c r="I28" s="11" t="n">
+        <v>1.226215045406112</v>
+      </c>
+      <c r="J28" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>IEF</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D29" s="11" t="n">
+        <v>0.03370980958751302</v>
+      </c>
+      <c r="E29" s="11" t="n">
+        <v>0.06790048151209217</v>
+      </c>
+      <c r="F29" s="10" t="n">
+        <v>0.522240288683088</v>
+      </c>
+      <c r="G29" s="10" t="n">
+        <v>0.7983896659541889</v>
+      </c>
+      <c r="H29" s="11" t="n">
+        <v>-0.2392477452272798</v>
+      </c>
+      <c r="I29" s="11" t="n">
+        <v>1.226215045406112</v>
+      </c>
+      <c r="J29" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N29" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>IEF</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D30" s="11" t="n">
+        <v>0.03370980958751302</v>
+      </c>
+      <c r="E30" s="11" t="n">
+        <v>0.06790048151209217</v>
+      </c>
+      <c r="F30" s="10" t="n">
+        <v>0.522240288683088</v>
+      </c>
+      <c r="G30" s="10" t="n">
+        <v>0.7983896659541889</v>
+      </c>
+      <c r="H30" s="11" t="n">
+        <v>-0.2392477452272798</v>
+      </c>
+      <c r="I30" s="11" t="n">
+        <v>1.226215045406112</v>
+      </c>
+      <c r="J30" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M30" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N30" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t>IEF</t>
+        </is>
+      </c>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C31" s="10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D31" s="11" t="n">
+        <v>0.03370980958751302</v>
+      </c>
+      <c r="E31" s="11" t="n">
+        <v>0.06790048151209217</v>
+      </c>
+      <c r="F31" s="10" t="n">
+        <v>0.522240288683088</v>
+      </c>
+      <c r="G31" s="10" t="n">
+        <v>0.7983896659541889</v>
+      </c>
+      <c r="H31" s="11" t="n">
+        <v>-0.2392477452272798</v>
+      </c>
+      <c r="I31" s="11" t="n">
+        <v>1.226215045406112</v>
+      </c>
+      <c r="J31" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M31" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N31" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>IEF</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D32" s="11" t="n">
+        <v>0.03370980958751302</v>
+      </c>
+      <c r="E32" s="11" t="n">
+        <v>0.06790048151209217</v>
+      </c>
+      <c r="F32" s="10" t="n">
+        <v>0.522240288683088</v>
+      </c>
+      <c r="G32" s="10" t="n">
+        <v>0.7983896659541889</v>
+      </c>
+      <c r="H32" s="11" t="n">
+        <v>-0.2392477452272798</v>
+      </c>
+      <c r="I32" s="11" t="n">
+        <v>1.226215045406112</v>
+      </c>
+      <c r="J32" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M32" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N32" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>IEF</t>
+        </is>
+      </c>
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t>trailing</t>
+        </is>
+      </c>
+      <c r="C33" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D33" s="11" t="n">
+        <v>0.03343681343503535</v>
+      </c>
+      <c r="E33" s="11" t="n">
+        <v>0.06767516380785676</v>
+      </c>
+      <c r="F33" s="10" t="n">
+        <v>0.5198498647550877</v>
+      </c>
+      <c r="G33" s="10" t="n">
+        <v>0.7928023929527597</v>
+      </c>
+      <c r="H33" s="11" t="n">
+        <v>-0.2440826956053245</v>
+      </c>
+      <c r="I33" s="11" t="n">
+        <v>1.212066366637341</v>
+      </c>
+      <c r="J33" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="K33" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="L33" s="11" t="n">
+        <v>0.006745426963743695</v>
+      </c>
+      <c r="M33" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N33" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
+          <t>IEF</t>
+        </is>
+      </c>
+      <c r="B34" s="10" t="inlineStr">
+        <is>
+          <t>trailing</t>
+        </is>
+      </c>
+      <c r="C34" s="10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D34" s="11" t="n">
+        <v>0.03409216599056109</v>
+      </c>
+      <c r="E34" s="11" t="n">
+        <v>0.06749965351020441</v>
+      </c>
+      <c r="F34" s="10" t="n">
+        <v>0.5304213757019554</v>
+      </c>
+      <c r="G34" s="10" t="n">
+        <v>0.8070989716799091</v>
+      </c>
+      <c r="H34" s="11" t="n">
+        <v>-0.232426088418173</v>
+      </c>
+      <c r="I34" s="11" t="n">
+        <v>1.246177490377855</v>
+      </c>
+      <c r="J34" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="K34" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="L34" s="11" t="n">
+        <v>-0.008277032074571311</v>
+      </c>
+      <c r="M34" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N34" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="inlineStr">
+        <is>
+          <t>IEF</t>
+        </is>
+      </c>
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>trailing</t>
+        </is>
+      </c>
+      <c r="C35" s="10" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D35" s="11" t="n">
+        <v>0.03370980958751302</v>
+      </c>
+      <c r="E35" s="11" t="n">
+        <v>0.06790048151209217</v>
+      </c>
+      <c r="F35" s="10" t="n">
+        <v>0.522240288683088</v>
+      </c>
+      <c r="G35" s="10" t="n">
+        <v>0.7983896659541889</v>
+      </c>
+      <c r="H35" s="11" t="n">
+        <v>-0.2392477452272798</v>
+      </c>
+      <c r="I35" s="11" t="n">
+        <v>1.226215045406112</v>
+      </c>
+      <c r="J35" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M35" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N35" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t>SHY</t>
+        </is>
+      </c>
+      <c r="B36" s="10" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="C36" s="10" t="n">
+        <v/>
+      </c>
+      <c r="D36" s="11" t="n">
+        <v>0.01960487657989041</v>
+      </c>
+      <c r="E36" s="11" t="n">
+        <v>0.01521116913279099</v>
+      </c>
+      <c r="F36" s="10" t="n">
+        <v>1.284027935849295</v>
+      </c>
+      <c r="G36" s="10" t="n">
+        <v>1.799783266370657</v>
+      </c>
+      <c r="H36" s="11" t="n">
+        <v>-0.05707117672507322</v>
+      </c>
+      <c r="I36" s="11" t="n">
+        <v>0.5979760006955412</v>
+      </c>
+      <c r="J36" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M36" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N36" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>SHY</t>
+        </is>
+      </c>
+      <c r="B37" s="10" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C37" s="10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D37" s="11" t="n">
+        <v>0.01960813086890423</v>
+      </c>
+      <c r="E37" s="11" t="n">
+        <v>0.01521241140635071</v>
+      </c>
+      <c r="F37" s="10" t="n">
+        <v>1.284134147174996</v>
+      </c>
+      <c r="G37" s="10" t="n">
+        <v>1.800079137366279</v>
+      </c>
+      <c r="H37" s="11" t="n">
+        <v>-0.05707117672507322</v>
+      </c>
+      <c r="I37" s="11" t="n">
+        <v>0.5979760006955412</v>
+      </c>
+      <c r="J37" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L37" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M37" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N37" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>SHY</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C38" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D38" s="11" t="n">
+        <v>0.01960813086890423</v>
+      </c>
+      <c r="E38" s="11" t="n">
+        <v>0.01521241140635071</v>
+      </c>
+      <c r="F38" s="10" t="n">
+        <v>1.284134147174996</v>
+      </c>
+      <c r="G38" s="10" t="n">
+        <v>1.800079137366279</v>
+      </c>
+      <c r="H38" s="11" t="n">
+        <v>-0.05707117672507322</v>
+      </c>
+      <c r="I38" s="11" t="n">
+        <v>0.5979760006955412</v>
+      </c>
+      <c r="J38" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K38" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L38" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M38" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N38" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t>SHY</t>
+        </is>
+      </c>
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C39" s="10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D39" s="11" t="n">
+        <v>0.01960813086890423</v>
+      </c>
+      <c r="E39" s="11" t="n">
+        <v>0.01521241140635071</v>
+      </c>
+      <c r="F39" s="10" t="n">
+        <v>1.284134147174996</v>
+      </c>
+      <c r="G39" s="10" t="n">
+        <v>1.800079137366279</v>
+      </c>
+      <c r="H39" s="11" t="n">
+        <v>-0.05707117672507322</v>
+      </c>
+      <c r="I39" s="11" t="n">
+        <v>0.5979760006955412</v>
+      </c>
+      <c r="J39" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K39" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L39" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M39" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N39" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="inlineStr">
+        <is>
+          <t>SHY</t>
+        </is>
+      </c>
+      <c r="B40" s="10" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C40" s="10" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D40" s="11" t="n">
+        <v>0.01960813086890423</v>
+      </c>
+      <c r="E40" s="11" t="n">
+        <v>0.01521241140635071</v>
+      </c>
+      <c r="F40" s="10" t="n">
+        <v>1.284134147174996</v>
+      </c>
+      <c r="G40" s="10" t="n">
+        <v>1.800079137366279</v>
+      </c>
+      <c r="H40" s="11" t="n">
+        <v>-0.05707117672507322</v>
+      </c>
+      <c r="I40" s="11" t="n">
+        <v>0.5979760006955412</v>
+      </c>
+      <c r="J40" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L40" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M40" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N40" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="10" t="inlineStr">
+        <is>
+          <t>SHY</t>
+        </is>
+      </c>
+      <c r="B41" s="10" t="inlineStr">
+        <is>
+          <t>trailing</t>
+        </is>
+      </c>
+      <c r="C41" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D41" s="11" t="n">
+        <v>0.01960813086890423</v>
+      </c>
+      <c r="E41" s="11" t="n">
+        <v>0.01521241140635071</v>
+      </c>
+      <c r="F41" s="10" t="n">
+        <v>1.284134147174996</v>
+      </c>
+      <c r="G41" s="10" t="n">
+        <v>1.800079137366279</v>
+      </c>
+      <c r="H41" s="11" t="n">
+        <v>-0.05707117672507322</v>
+      </c>
+      <c r="I41" s="11" t="n">
+        <v>0.5979760006955412</v>
+      </c>
+      <c r="J41" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L41" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M41" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N41" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="inlineStr">
+        <is>
+          <t>SHY</t>
+        </is>
+      </c>
+      <c r="B42" s="10" t="inlineStr">
+        <is>
+          <t>trailing</t>
+        </is>
+      </c>
+      <c r="C42" s="10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D42" s="11" t="n">
+        <v>0.01960813086890423</v>
+      </c>
+      <c r="E42" s="11" t="n">
+        <v>0.01521241140635071</v>
+      </c>
+      <c r="F42" s="10" t="n">
+        <v>1.284134147174996</v>
+      </c>
+      <c r="G42" s="10" t="n">
+        <v>1.800079137366279</v>
+      </c>
+      <c r="H42" s="11" t="n">
+        <v>-0.05707117672507322</v>
+      </c>
+      <c r="I42" s="11" t="n">
+        <v>0.5979760006955412</v>
+      </c>
+      <c r="J42" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K42" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L42" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M42" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N42" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="10" t="inlineStr">
+        <is>
+          <t>SHY</t>
+        </is>
+      </c>
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>trailing</t>
+        </is>
+      </c>
+      <c r="C43" s="10" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D43" s="11" t="n">
+        <v>0.01960813086890423</v>
+      </c>
+      <c r="E43" s="11" t="n">
+        <v>0.01521241140635071</v>
+      </c>
+      <c r="F43" s="10" t="n">
+        <v>1.284134147174996</v>
+      </c>
+      <c r="G43" s="10" t="n">
+        <v>1.800079137366279</v>
+      </c>
+      <c r="H43" s="11" t="n">
+        <v>-0.05707117672507322</v>
+      </c>
+      <c r="I43" s="11" t="n">
+        <v>0.5979760006955412</v>
+      </c>
+      <c r="J43" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K43" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L43" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M43" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N43" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="inlineStr">
+        <is>
+          <t>VOO</t>
+        </is>
+      </c>
+      <c r="B44" s="10" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="C44" s="10" t="n">
+        <v/>
+      </c>
+      <c r="D44" s="11" t="n">
+        <v>0.1491637107584858</v>
+      </c>
+      <c r="E44" s="11" t="n">
+        <v>0.1695279537052974</v>
+      </c>
+      <c r="F44" s="10" t="n">
+        <v>0.9053509047751095</v>
+      </c>
+      <c r="G44" s="10" t="n">
+        <v>1.113627117737396</v>
+      </c>
+      <c r="H44" s="11" t="n">
+        <v>-0.3399302268072862</v>
+      </c>
+      <c r="I44" s="11" t="n">
+        <v>8.295375640156196</v>
+      </c>
+      <c r="J44" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L44" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M44" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N44" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="10" t="inlineStr">
+        <is>
+          <t>VOO</t>
+        </is>
+      </c>
+      <c r="B45" s="10" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C45" s="10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D45" s="11" t="n">
+        <v>0.1492032593021795</v>
+      </c>
+      <c r="E45" s="11" t="n">
+        <v>0.1695488705143411</v>
+      </c>
+      <c r="F45" s="10" t="n">
+        <v>0.9054632830697465</v>
+      </c>
+      <c r="G45" s="10" t="n">
+        <v>1.113902768014063</v>
+      </c>
+      <c r="H45" s="11" t="n">
+        <v>-0.3399302268072862</v>
+      </c>
+      <c r="I45" s="11" t="n">
+        <v>8.295375640156196</v>
+      </c>
+      <c r="J45" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L45" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M45" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N45" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="10" t="inlineStr">
+        <is>
+          <t>VOO</t>
+        </is>
+      </c>
+      <c r="B46" s="10" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C46" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D46" s="11" t="n">
+        <v>0.1492032593021795</v>
+      </c>
+      <c r="E46" s="11" t="n">
+        <v>0.1695488705143411</v>
+      </c>
+      <c r="F46" s="10" t="n">
+        <v>0.9054632830697465</v>
+      </c>
+      <c r="G46" s="10" t="n">
+        <v>1.113902768014063</v>
+      </c>
+      <c r="H46" s="11" t="n">
+        <v>-0.3399302268072862</v>
+      </c>
+      <c r="I46" s="11" t="n">
+        <v>8.295375640156196</v>
+      </c>
+      <c r="J46" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L46" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M46" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N46" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="10" t="inlineStr">
+        <is>
+          <t>VOO</t>
+        </is>
+      </c>
+      <c r="B47" s="10" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C47" s="10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D47" s="11" t="n">
+        <v>0.1492032593021795</v>
+      </c>
+      <c r="E47" s="11" t="n">
+        <v>0.1695488705143411</v>
+      </c>
+      <c r="F47" s="10" t="n">
+        <v>0.9054632830697465</v>
+      </c>
+      <c r="G47" s="10" t="n">
+        <v>1.113902768014063</v>
+      </c>
+      <c r="H47" s="11" t="n">
+        <v>-0.3399302268072862</v>
+      </c>
+      <c r="I47" s="11" t="n">
+        <v>8.295375640156196</v>
+      </c>
+      <c r="J47" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K47" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L47" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M47" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N47" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="10" t="inlineStr">
+        <is>
+          <t>VOO</t>
+        </is>
+      </c>
+      <c r="B48" s="10" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="C48" s="10" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D48" s="11" t="n">
+        <v>0.1492032593021795</v>
+      </c>
+      <c r="E48" s="11" t="n">
+        <v>0.1695488705143411</v>
+      </c>
+      <c r="F48" s="10" t="n">
+        <v>0.9054632830697465</v>
+      </c>
+      <c r="G48" s="10" t="n">
+        <v>1.113902768014063</v>
+      </c>
+      <c r="H48" s="11" t="n">
+        <v>-0.3399302268072862</v>
+      </c>
+      <c r="I48" s="11" t="n">
+        <v>8.295375640156196</v>
+      </c>
+      <c r="J48" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K48" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L48" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M48" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N48" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="10" t="inlineStr">
+        <is>
+          <t>VOO</t>
+        </is>
+      </c>
+      <c r="B49" s="10" t="inlineStr">
+        <is>
+          <t>trailing</t>
+        </is>
+      </c>
+      <c r="C49" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D49" s="11" t="n">
+        <v>0.1285991559350201</v>
+      </c>
+      <c r="E49" s="11" t="n">
+        <v>0.1471697169194991</v>
+      </c>
+      <c r="F49" s="10" t="n">
+        <v>0.8960892661056504</v>
+      </c>
+      <c r="G49" s="10" t="n">
+        <v>1.098844790427607</v>
+      </c>
+      <c r="H49" s="11" t="n">
+        <v>-0.2771448011146757</v>
+      </c>
+      <c r="I49" s="11" t="n">
+        <v>5.955101395132457</v>
+      </c>
+      <c r="J49" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K49" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="L49" s="11" t="n">
+        <v>0.3469762546413566</v>
+      </c>
+      <c r="M49" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N49" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="10" t="inlineStr">
+        <is>
+          <t>VOO</t>
+        </is>
+      </c>
+      <c r="B50" s="10" t="inlineStr">
+        <is>
+          <t>trailing</t>
+        </is>
+      </c>
+      <c r="C50" s="10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D50" s="11" t="n">
+        <v>0.1403355589744564</v>
+      </c>
+      <c r="E50" s="11" t="n">
+        <v>0.1580223448829602</v>
+      </c>
+      <c r="F50" s="10" t="n">
+        <v>0.910542035463991</v>
+      </c>
+      <c r="G50" s="10" t="n">
+        <v>1.12136614762773</v>
+      </c>
+      <c r="H50" s="11" t="n">
+        <v>-0.2746363913759123</v>
+      </c>
+      <c r="I50" s="11" t="n">
+        <v>7.209812421105982</v>
+      </c>
+      <c r="J50" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="K50" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="L50" s="11" t="n">
+        <v>0.1544544805069981</v>
+      </c>
+      <c r="M50" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N50" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="10" t="inlineStr">
+        <is>
+          <t>VOO</t>
+        </is>
+      </c>
+      <c r="B51" s="10" t="inlineStr">
+        <is>
+          <t>trailing</t>
+        </is>
+      </c>
+      <c r="C51" s="10" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D51" s="11" t="n">
+        <v>0.1412395085149012</v>
+      </c>
+      <c r="E51" s="11" t="n">
+        <v>0.1588272107280826</v>
+      </c>
+      <c r="F51" s="10" t="n">
+        <v>0.9117224171114825</v>
+      </c>
+      <c r="G51" s="10" t="n">
+        <v>1.127076136702849</v>
+      </c>
+      <c r="H51" s="11" t="n">
+        <v>-0.2746363913759123</v>
+      </c>
+      <c r="I51" s="11" t="n">
+        <v>7.314770272941587</v>
+      </c>
+      <c r="J51" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="K51" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="L51" s="11" t="n">
+        <v>0.1396998087823249</v>
+      </c>
+      <c r="M51" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="N51" s="10" t="inlineStr">
+        <is>
+          <t>Historical backtest on adjusted prices; re-entry after 21 trading days. Not a recommendation to adopt any stop.</t>
         </is>
       </c>
     </row>
@@ -6226,7 +8737,7 @@
     <col width="24" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
@@ -6332,10 +8843,10 @@
         </is>
       </c>
       <c r="J4" s="11" t="n">
-        <v/>
+        <v>0.355327691196202</v>
       </c>
       <c r="K4" s="11" t="n">
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -6375,10 +8886,10 @@
         </is>
       </c>
       <c r="J5" s="11" t="n">
-        <v/>
+        <v>0.09467230880379809</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -6418,10 +8929,10 @@
         </is>
       </c>
       <c r="J6" s="11" t="n">
-        <v/>
+        <v>0.25</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -6461,10 +8972,10 @@
         </is>
       </c>
       <c r="J7" s="11" t="n">
-        <v/>
+        <v>0.175</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -6504,10 +9015,10 @@
         </is>
       </c>
       <c r="J8" s="11" t="n">
-        <v/>
+        <v>0.125</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v/>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Surface capital-floor probabilities, inflation scenarios, and drawdown recovery events in Risk sheet
</commit_message>
<xml_diff>
--- a/portfolio_model/outputs/spreadsheet/portfolio_analysis.xlsx
+++ b/portfolio_model/outputs/spreadsheet/portfolio_analysis.xlsx
@@ -33,9 +33,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -125,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -144,6 +145,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -525,7 +527,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-04 18:50 UTC | Seed: 42 | Simulations: 10000 | Model version: 1.0.0</t>
+          <t>Generated: 2026-10-04 18:51 UTC | Seed: 42 | Simulations: 10000 | Model version: 1.0.0</t>
         </is>
       </c>
     </row>
@@ -3326,11 +3328,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="33" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3581,6 +3586,687 @@
       </c>
       <c r="B26" s="11" t="n">
         <v>0.2041</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>MC success above real capital @ 2% inflation</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="n">
+        <v>0.8485</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>Bootstrap success above real capital @ 2% inflation</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="n">
+        <v>0.8679</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>MC success above real capital @ 3% inflation</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="n">
+        <v>0.7921</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>Bootstrap success above real capital @ 3% inflation</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="n">
+        <v>0.8125</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t>MC success above real capital @ 4% inflation</t>
+        </is>
+      </c>
+      <c r="B31" s="11" t="n">
+        <v>0.7271</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>Bootstrap success above real capital @ 4% inflation</t>
+        </is>
+      </c>
+      <c r="B32" s="11" t="n">
+        <v>0.7483</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>MC success above real capital @ 5% inflation</t>
+        </is>
+      </c>
+      <c r="B33" s="11" t="n">
+        <v>0.6552</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
+          <t>Bootstrap success above real capital @ 5% inflation</t>
+        </is>
+      </c>
+      <c r="B34" s="11" t="n">
+        <v>0.6771</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="inlineStr">
+        <is>
+          <t>MC prob terminal above 100% real capital floor</t>
+        </is>
+      </c>
+      <c r="B35" s="11" t="n">
+        <v>0.8485</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t>MC prob terminal above 90% real capital floor</t>
+        </is>
+      </c>
+      <c r="B36" s="11" t="n">
+        <v>0.9179</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>MC prob terminal above 80% real capital floor</t>
+        </is>
+      </c>
+      <c r="B37" s="11" t="n">
+        <v>0.9651999999999999</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>MC prob terminal above 70% real capital floor</t>
+        </is>
+      </c>
+      <c r="B38" s="11" t="n">
+        <v>0.9898</v>
+      </c>
+    </row>
+    <row r="39"/>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>Major Drawdown Recovery Events</t>
+        </is>
+      </c>
+    </row>
+    <row r="41"/>
+    <row r="42">
+      <c r="A42" s="9" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>trough</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>drawdown</t>
+        </is>
+      </c>
+      <c r="D42" s="9" t="inlineStr">
+        <is>
+          <t>recovery</t>
+        </is>
+      </c>
+      <c r="E42" s="9" t="inlineStr">
+        <is>
+          <t>days_to_recover</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="10" t="inlineStr">
+        <is>
+          <t>2000-02-24</t>
+        </is>
+      </c>
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>2000-03-08</t>
+        </is>
+      </c>
+      <c r="C43" s="11" t="n">
+        <v>-0.0521921011703137</v>
+      </c>
+      <c r="D43" s="10" t="inlineStr">
+        <is>
+          <t>2000-03-22</t>
+        </is>
+      </c>
+      <c r="E43" s="10" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="inlineStr">
+        <is>
+          <t>2000-04-07</t>
+        </is>
+      </c>
+      <c r="B44" s="10" t="inlineStr">
+        <is>
+          <t>2000-04-14</t>
+        </is>
+      </c>
+      <c r="C44" s="11" t="n">
+        <v>-0.05466104755209877</v>
+      </c>
+      <c r="D44" s="10" t="inlineStr">
+        <is>
+          <t>2000-04-27</t>
+        </is>
+      </c>
+      <c r="E44" s="10" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="10" t="inlineStr">
+        <is>
+          <t>2000-05-01</t>
+        </is>
+      </c>
+      <c r="B45" s="10" t="inlineStr">
+        <is>
+          <t>2000-05-26</t>
+        </is>
+      </c>
+      <c r="C45" s="11" t="n">
+        <v>-0.05127731982185779</v>
+      </c>
+      <c r="D45" s="10" t="inlineStr">
+        <is>
+          <t>2000-06-05</t>
+        </is>
+      </c>
+      <c r="E45" s="10" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="10" t="inlineStr">
+        <is>
+          <t>2000-10-03</t>
+        </is>
+      </c>
+      <c r="B46" s="10" t="inlineStr">
+        <is>
+          <t>2000-10-18</t>
+        </is>
+      </c>
+      <c r="C46" s="11" t="n">
+        <v>-0.05563111409934318</v>
+      </c>
+      <c r="D46" s="10" t="inlineStr">
+        <is>
+          <t>2000-11-03</t>
+        </is>
+      </c>
+      <c r="E46" s="10" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="10" t="inlineStr">
+        <is>
+          <t>2000-11-06</t>
+        </is>
+      </c>
+      <c r="B47" s="10" t="inlineStr">
+        <is>
+          <t>2002-08-05</t>
+        </is>
+      </c>
+      <c r="C47" s="11" t="n">
+        <v>-0.2738278820192828</v>
+      </c>
+      <c r="D47" s="10" t="inlineStr">
+        <is>
+          <t>2004-04-08</t>
+        </is>
+      </c>
+      <c r="E47" s="10" t="n">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="10" t="inlineStr">
+        <is>
+          <t>2005-04-07</t>
+        </is>
+      </c>
+      <c r="B48" s="10" t="inlineStr">
+        <is>
+          <t>2005-08-10</t>
+        </is>
+      </c>
+      <c r="C48" s="11" t="n">
+        <v>-0.06324292035717383</v>
+      </c>
+      <c r="D48" s="10" t="inlineStr">
+        <is>
+          <t>2005-11-17</t>
+        </is>
+      </c>
+      <c r="E48" s="10" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="10" t="inlineStr">
+        <is>
+          <t>2006-04-27</t>
+        </is>
+      </c>
+      <c r="B49" s="10" t="inlineStr">
+        <is>
+          <t>2006-07-27</t>
+        </is>
+      </c>
+      <c r="C49" s="11" t="n">
+        <v>-0.07428113354669819</v>
+      </c>
+      <c r="D49" s="10" t="inlineStr">
+        <is>
+          <t>2006-09-15</t>
+        </is>
+      </c>
+      <c r="E49" s="10" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="10" t="inlineStr">
+        <is>
+          <t>2007-10-24</t>
+        </is>
+      </c>
+      <c r="B50" s="10" t="inlineStr">
+        <is>
+          <t>2008-03-17</t>
+        </is>
+      </c>
+      <c r="C50" s="11" t="n">
+        <v>-0.08861883761513201</v>
+      </c>
+      <c r="D50" s="10" t="inlineStr">
+        <is>
+          <t>2008-08-08</t>
+        </is>
+      </c>
+      <c r="E50" s="10" t="n">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="10" t="inlineStr">
+        <is>
+          <t>2008-08-11</t>
+        </is>
+      </c>
+      <c r="B51" s="10" t="inlineStr">
+        <is>
+          <t>2009-03-02</t>
+        </is>
+      </c>
+      <c r="C51" s="11" t="n">
+        <v>-0.2234914167744868</v>
+      </c>
+      <c r="D51" s="10" t="inlineStr">
+        <is>
+          <t>2009-10-19</t>
+        </is>
+      </c>
+      <c r="E51" s="10" t="n">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="10" t="inlineStr">
+        <is>
+          <t>2010-04-26</t>
+        </is>
+      </c>
+      <c r="B52" s="10" t="inlineStr">
+        <is>
+          <t>2010-07-06</t>
+        </is>
+      </c>
+      <c r="C52" s="11" t="n">
+        <v>-0.0727702413546627</v>
+      </c>
+      <c r="D52" s="10" t="inlineStr">
+        <is>
+          <t>2010-11-04</t>
+        </is>
+      </c>
+      <c r="E52" s="10" t="n">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="10" t="inlineStr">
+        <is>
+          <t>2011-05-12</t>
+        </is>
+      </c>
+      <c r="B53" s="10" t="inlineStr">
+        <is>
+          <t>2011-10-03</t>
+        </is>
+      </c>
+      <c r="C53" s="11" t="n">
+        <v>-0.151462881549703</v>
+      </c>
+      <c r="D53" s="10" t="inlineStr">
+        <is>
+          <t>2012-02-07</t>
+        </is>
+      </c>
+      <c r="E53" s="10" t="n">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="10" t="inlineStr">
+        <is>
+          <t>2012-04-02</t>
+        </is>
+      </c>
+      <c r="B54" s="10" t="inlineStr">
+        <is>
+          <t>2012-06-01</t>
+        </is>
+      </c>
+      <c r="C54" s="11" t="n">
+        <v>-0.05134607162890448</v>
+      </c>
+      <c r="D54" s="10" t="inlineStr">
+        <is>
+          <t>2012-08-07</t>
+        </is>
+      </c>
+      <c r="E54" s="10" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="10" t="inlineStr">
+        <is>
+          <t>2014-09-05</t>
+        </is>
+      </c>
+      <c r="B55" s="10" t="inlineStr">
+        <is>
+          <t>2014-10-14</t>
+        </is>
+      </c>
+      <c r="C55" s="11" t="n">
+        <v>-0.05901319257984405</v>
+      </c>
+      <c r="D55" s="10" t="inlineStr">
+        <is>
+          <t>2014-11-05</t>
+        </is>
+      </c>
+      <c r="E55" s="10" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="10" t="inlineStr">
+        <is>
+          <t>2015-08-17</t>
+        </is>
+      </c>
+      <c r="B56" s="10" t="inlineStr">
+        <is>
+          <t>2015-08-25</t>
+        </is>
+      </c>
+      <c r="C56" s="11" t="n">
+        <v>-0.07105828209581821</v>
+      </c>
+      <c r="D56" s="10" t="inlineStr">
+        <is>
+          <t>2015-10-16</t>
+        </is>
+      </c>
+      <c r="E56" s="10" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="10" t="inlineStr">
+        <is>
+          <t>2015-12-16</t>
+        </is>
+      </c>
+      <c r="B57" s="10" t="inlineStr">
+        <is>
+          <t>2016-02-11</t>
+        </is>
+      </c>
+      <c r="C57" s="11" t="n">
+        <v>-0.09453428136673914</v>
+      </c>
+      <c r="D57" s="10" t="inlineStr">
+        <is>
+          <t>2016-04-18</t>
+        </is>
+      </c>
+      <c r="E57" s="10" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="10" t="inlineStr">
+        <is>
+          <t>2018-01-26</t>
+        </is>
+      </c>
+      <c r="B58" s="10" t="inlineStr">
+        <is>
+          <t>2018-02-08</t>
+        </is>
+      </c>
+      <c r="C58" s="11" t="n">
+        <v>-0.05294273580221653</v>
+      </c>
+      <c r="D58" s="10" t="inlineStr">
+        <is>
+          <t>2018-02-26</t>
+        </is>
+      </c>
+      <c r="E58" s="10" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="10" t="inlineStr">
+        <is>
+          <t>2018-10-01</t>
+        </is>
+      </c>
+      <c r="B59" s="10" t="inlineStr">
+        <is>
+          <t>2018-12-24</t>
+        </is>
+      </c>
+      <c r="C59" s="11" t="n">
+        <v>-0.1149527575798448</v>
+      </c>
+      <c r="D59" s="10" t="inlineStr">
+        <is>
+          <t>2019-04-01</t>
+        </is>
+      </c>
+      <c r="E59" s="10" t="n">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="10" t="inlineStr">
+        <is>
+          <t>2020-02-19</t>
+        </is>
+      </c>
+      <c r="B60" s="10" t="inlineStr">
+        <is>
+          <t>2020-03-20</t>
+        </is>
+      </c>
+      <c r="C60" s="11" t="n">
+        <v>-0.1676653273065402</v>
+      </c>
+      <c r="D60" s="10" t="inlineStr">
+        <is>
+          <t>2020-06-05</t>
+        </is>
+      </c>
+      <c r="E60" s="10" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="10" t="inlineStr">
+        <is>
+          <t>2020-09-02</t>
+        </is>
+      </c>
+      <c r="B61" s="10" t="inlineStr">
+        <is>
+          <t>2020-10-30</t>
+        </is>
+      </c>
+      <c r="C61" s="11" t="n">
+        <v>-0.06650427186097196</v>
+      </c>
+      <c r="D61" s="10" t="inlineStr">
+        <is>
+          <t>2020-12-02</t>
+        </is>
+      </c>
+      <c r="E61" s="10" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="10" t="inlineStr">
+        <is>
+          <t>2021-09-16</t>
+        </is>
+      </c>
+      <c r="B62" s="10" t="inlineStr">
+        <is>
+          <t>2022-10-14</t>
+        </is>
+      </c>
+      <c r="C62" s="11" t="n">
+        <v>-0.3102036234978799</v>
+      </c>
+      <c r="D62" s="10" t="inlineStr">
+        <is>
+          <t>2023-11-09</t>
+        </is>
+      </c>
+      <c r="E62" s="10" t="n">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="10" t="inlineStr">
+        <is>
+          <t>2024-03-12</t>
+        </is>
+      </c>
+      <c r="B63" s="10" t="inlineStr">
+        <is>
+          <t>2024-08-05</t>
+        </is>
+      </c>
+      <c r="C63" s="11" t="n">
+        <v>-0.07557404153182967</v>
+      </c>
+      <c r="D63" s="10" t="inlineStr">
+        <is>
+          <t>2024-08-19</t>
+        </is>
+      </c>
+      <c r="E63" s="10" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="10" t="inlineStr">
+        <is>
+          <t>2024-12-06</t>
+        </is>
+      </c>
+      <c r="B64" s="10" t="inlineStr">
+        <is>
+          <t>2025-04-08</t>
+        </is>
+      </c>
+      <c r="C64" s="11" t="n">
+        <v>-0.1835251727933562</v>
+      </c>
+      <c r="D64" s="10" t="inlineStr">
+        <is>
+          <t>2025-05-16</t>
+        </is>
+      </c>
+      <c r="E64" s="10" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="10" t="inlineStr">
+        <is>
+          <t>2025-05-16</t>
+        </is>
+      </c>
+      <c r="B65" s="10" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C65" s="11" t="n">
+        <v>-0.2729570297725958</v>
+      </c>
+      <c r="D65" s="16" t="n"/>
+      <c r="E65" s="10" t="n">
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -4729,308 +5415,308 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="17" t="inlineStr">
         <is>
           <t>ADBE,DIS,DUOL,VOO</t>
         </is>
       </c>
-      <c r="C4" s="16" t="inlineStr">
+      <c r="C4" s="17" t="inlineStr">
         <is>
           <t>Missing sector</t>
         </is>
       </c>
-      <c r="D4" s="16" t="inlineStr">
+      <c r="D4" s="17" t="inlineStr">
         <is>
           <t>Sector will be assigned via classification lookup.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>Growth/Consumer-Tech</t>
         </is>
       </c>
-      <c r="C5" s="16" t="inlineStr">
+      <c r="C5" s="17" t="inlineStr">
         <is>
           <t>CORRELATED-GROUP OVERWEIGHT</t>
         </is>
       </c>
-      <c r="D5" s="16" t="inlineStr">
+      <c r="D5" s="17" t="inlineStr">
         <is>
           <t>Group 'Growth/Consumer-Tech' totals 45.0% &gt; cap 30%.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>info</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>ADBE</t>
         </is>
       </c>
-      <c r="C6" s="16" t="inlineStr">
+      <c r="C6" s="17" t="inlineStr">
         <is>
           <t>Data status</t>
         </is>
       </c>
-      <c r="D6" s="16" t="inlineStr">
-        <is>
-          <t>{'status': 'ok', 'inception': '2000-01-03', 'rows': 6728, 'fetched_utc': '2026-10-04T18:50:25.797519+00:00'}</t>
+      <c r="D6" s="17" t="inlineStr">
+        <is>
+          <t>{'status': 'ok', 'inception': '2000-01-03', 'rows': 6728, 'fetched_utc': '2026-10-04T18:51:43.507137+00:00'}</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>info</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>DIS</t>
         </is>
       </c>
-      <c r="C7" s="16" t="inlineStr">
+      <c r="C7" s="17" t="inlineStr">
         <is>
           <t>Data status</t>
         </is>
       </c>
-      <c r="D7" s="16" t="inlineStr">
-        <is>
-          <t>{'status': 'ok', 'inception': '2000-01-03', 'rows': 6728, 'fetched_utc': '2026-10-04T18:50:25.800034+00:00'}</t>
+      <c r="D7" s="17" t="inlineStr">
+        <is>
+          <t>{'status': 'ok', 'inception': '2000-01-03', 'rows': 6728, 'fetched_utc': '2026-10-04T18:51:43.509362+00:00'}</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>info</t>
         </is>
       </c>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>DUOL</t>
         </is>
       </c>
-      <c r="C8" s="16" t="inlineStr">
+      <c r="C8" s="17" t="inlineStr">
         <is>
           <t>Data status</t>
         </is>
       </c>
-      <c r="D8" s="16" t="inlineStr">
-        <is>
-          <t>{'status': 'ok', 'inception': '2021-07-28', 'rows': 1302, 'fetched_utc': '2026-10-04T18:50:25.801697+00:00'}</t>
+      <c r="D8" s="17" t="inlineStr">
+        <is>
+          <t>{'status': 'ok', 'inception': '2021-07-28', 'rows': 1302, 'fetched_utc': '2026-10-04T18:51:43.511320+00:00'}</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>info</t>
         </is>
       </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>IEF</t>
         </is>
       </c>
-      <c r="C9" s="16" t="inlineStr">
+      <c r="C9" s="17" t="inlineStr">
         <is>
           <t>Data status</t>
         </is>
       </c>
-      <c r="D9" s="16" t="inlineStr">
-        <is>
-          <t>{'status': 'ok', 'inception': '2002-07-30', 'rows': 6084, 'fetched_utc': '2026-10-04T18:50:25.803463+00:00'}</t>
+      <c r="D9" s="17" t="inlineStr">
+        <is>
+          <t>{'status': 'ok', 'inception': '2002-07-30', 'rows': 6084, 'fetched_utc': '2026-10-04T18:51:43.513118+00:00'}</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>info</t>
         </is>
       </c>
-      <c r="B10" s="16" t="inlineStr">
+      <c r="B10" s="17" t="inlineStr">
         <is>
           <t>SHY</t>
         </is>
       </c>
-      <c r="C10" s="16" t="inlineStr">
+      <c r="C10" s="17" t="inlineStr">
         <is>
           <t>Data status</t>
         </is>
       </c>
-      <c r="D10" s="16" t="inlineStr">
-        <is>
-          <t>{'status': 'ok', 'inception': '2002-07-30', 'rows': 6084, 'fetched_utc': '2026-10-04T18:50:25.805187+00:00'}</t>
+      <c r="D10" s="17" t="inlineStr">
+        <is>
+          <t>{'status': 'ok', 'inception': '2002-07-30', 'rows': 6084, 'fetched_utc': '2026-10-04T18:51:43.515281+00:00'}</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>info</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>VOO</t>
         </is>
       </c>
-      <c r="C11" s="16" t="inlineStr">
+      <c r="C11" s="17" t="inlineStr">
         <is>
           <t>Data status</t>
         </is>
       </c>
-      <c r="D11" s="16" t="inlineStr">
-        <is>
-          <t>{'status': 'ok', 'inception': '2010-09-09', 'rows': 4041, 'fetched_utc': '2026-10-04T18:50:25.806728+00:00'}</t>
+      <c r="D11" s="17" t="inlineStr">
+        <is>
+          <t>{'status': 'ok', 'inception': '2010-09-09', 'rows': 4041, 'fetched_utc': '2026-10-04T18:51:43.517393+00:00'}</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>info</t>
         </is>
       </c>
-      <c r="B12" s="16" t="inlineStr">
+      <c r="B12" s="17" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="C12" s="16" t="inlineStr">
+      <c r="C12" s="17" t="inlineStr">
         <is>
           <t>Data status</t>
         </is>
       </c>
-      <c r="D12" s="16" t="inlineStr">
-        <is>
-          <t>{'status': 'ok', 'inception': '2000-01-03', 'rows': 6728, 'fetched_utc': '2026-10-04T18:50:25.808489+00:00'}</t>
+      <c r="D12" s="17" t="inlineStr">
+        <is>
+          <t>{'status': 'ok', 'inception': '2000-01-03', 'rows': 6728, 'fetched_utc': '2026-10-04T18:51:43.519527+00:00'}</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="inlineStr">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>info</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="17" t="inlineStr">
         <is>
           <t>AGG</t>
         </is>
       </c>
-      <c r="C13" s="16" t="inlineStr">
+      <c r="C13" s="17" t="inlineStr">
         <is>
           <t>Data status</t>
         </is>
       </c>
-      <c r="D13" s="16" t="inlineStr">
-        <is>
-          <t>{'status': 'ok', 'inception': '2003-09-29', 'rows': 5790, 'fetched_utc': '2026-10-04T18:50:25.810154+00:00'}</t>
+      <c r="D13" s="17" t="inlineStr">
+        <is>
+          <t>{'status': 'ok', 'inception': '2003-09-29', 'rows': 5790, 'fetched_utc': '2026-10-04T18:51:43.521581+00:00'}</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="inlineStr">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>info</t>
         </is>
       </c>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="17" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C14" s="16" t="inlineStr">
+      <c r="C14" s="17" t="inlineStr">
         <is>
           <t>Survivorship bias</t>
         </is>
       </c>
-      <c r="D14" s="16" t="inlineStr">
+      <c r="D14" s="17" t="inlineStr">
         <is>
           <t>Historical analysis is subject to survivorship bias because securities that no longer exist are not represented.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>info</t>
         </is>
       </c>
-      <c r="B15" s="16" t="inlineStr">
+      <c r="B15" s="17" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C15" s="16" t="inlineStr">
+      <c r="C15" s="17" t="inlineStr">
         <is>
           <t>Returns basis</t>
         </is>
       </c>
-      <c r="D15" s="16" t="inlineStr">
+      <c r="D15" s="17" t="inlineStr">
         <is>
           <t>Adjusted close (dividend/total-return) prices used; returns include dividends.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="inlineStr">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>info</t>
         </is>
       </c>
-      <c r="B16" s="16" t="inlineStr">
+      <c r="B16" s="17" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C16" s="16" t="inlineStr">
+      <c r="C16" s="17" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
-      <c r="D16" s="16" t="inlineStr">
+      <c r="D16" s="17" t="inlineStr">
         <is>
           <t>Dollar P&amp;L is not computed because no cost basis / purchase price was supplied in the input spreadsheet. Return-based attribution is used instead (spec section 64: do not invent data).</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>info</t>
         </is>
       </c>
-      <c r="B17" s="16" t="inlineStr">
+      <c r="B17" s="17" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C17" s="16" t="inlineStr">
+      <c r="C17" s="17" t="inlineStr">
         <is>
           <t>Taxes</t>
         </is>
       </c>
-      <c r="D17" s="16" t="inlineStr">
+      <c r="D17" s="17" t="inlineStr">
         <is>
           <t>Tax effects are excluded because sufficient tax-lot information was not supplied.</t>
         </is>

</xml_diff>

<commit_message>
Harden spreadsheet uploads: numeric coercion, invalid/foreign ticker flags, currency exclusion, missing-weight errors, formula detection, minimal-column defaults, example inputs + format docs
</commit_message>
<xml_diff>
--- a/portfolio_model/outputs/spreadsheet/portfolio_analysis.xlsx
+++ b/portfolio_model/outputs/spreadsheet/portfolio_analysis.xlsx
@@ -527,7 +527,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-04 18:51 UTC | Seed: 42 | Simulations: 10000 | Model version: 1.0.0</t>
+          <t>Generated: 2026-10-04 19:22 UTC | Seed: 42 | Simulations: 10000 | Model version: 1.0.0</t>
         </is>
       </c>
     </row>
@@ -5476,7 +5476,7 @@
       </c>
       <c r="D6" s="17" t="inlineStr">
         <is>
-          <t>{'status': 'ok', 'inception': '2000-01-03', 'rows': 6728, 'fetched_utc': '2026-10-04T18:51:43.507137+00:00'}</t>
+          <t>{'status': 'ok', 'inception': '2000-01-03', 'rows': 6728, 'fetched_utc': '2026-10-04T19:22:06.849981+00:00'}</t>
         </is>
       </c>
     </row>
@@ -5498,7 +5498,7 @@
       </c>
       <c r="D7" s="17" t="inlineStr">
         <is>
-          <t>{'status': 'ok', 'inception': '2000-01-03', 'rows': 6728, 'fetched_utc': '2026-10-04T18:51:43.509362+00:00'}</t>
+          <t>{'status': 'ok', 'inception': '2000-01-03', 'rows': 6728, 'fetched_utc': '2026-10-04T19:22:06.852541+00:00'}</t>
         </is>
       </c>
     </row>
@@ -5520,7 +5520,7 @@
       </c>
       <c r="D8" s="17" t="inlineStr">
         <is>
-          <t>{'status': 'ok', 'inception': '2021-07-28', 'rows': 1302, 'fetched_utc': '2026-10-04T18:51:43.511320+00:00'}</t>
+          <t>{'status': 'ok', 'inception': '2021-07-28', 'rows': 1302, 'fetched_utc': '2026-10-04T19:22:06.854829+00:00'}</t>
         </is>
       </c>
     </row>
@@ -5542,7 +5542,7 @@
       </c>
       <c r="D9" s="17" t="inlineStr">
         <is>
-          <t>{'status': 'ok', 'inception': '2002-07-30', 'rows': 6084, 'fetched_utc': '2026-10-04T18:51:43.513118+00:00'}</t>
+          <t>{'status': 'ok', 'inception': '2002-07-30', 'rows': 6084, 'fetched_utc': '2026-10-04T19:22:06.857470+00:00'}</t>
         </is>
       </c>
     </row>
@@ -5564,7 +5564,7 @@
       </c>
       <c r="D10" s="17" t="inlineStr">
         <is>
-          <t>{'status': 'ok', 'inception': '2002-07-30', 'rows': 6084, 'fetched_utc': '2026-10-04T18:51:43.515281+00:00'}</t>
+          <t>{'status': 'ok', 'inception': '2002-07-30', 'rows': 6084, 'fetched_utc': '2026-10-04T19:22:06.861466+00:00'}</t>
         </is>
       </c>
     </row>
@@ -5586,7 +5586,7 @@
       </c>
       <c r="D11" s="17" t="inlineStr">
         <is>
-          <t>{'status': 'ok', 'inception': '2010-09-09', 'rows': 4041, 'fetched_utc': '2026-10-04T18:51:43.517393+00:00'}</t>
+          <t>{'status': 'ok', 'inception': '2010-09-09', 'rows': 4041, 'fetched_utc': '2026-10-04T19:22:06.863315+00:00'}</t>
         </is>
       </c>
     </row>
@@ -5608,7 +5608,7 @@
       </c>
       <c r="D12" s="17" t="inlineStr">
         <is>
-          <t>{'status': 'ok', 'inception': '2000-01-03', 'rows': 6728, 'fetched_utc': '2026-10-04T18:51:43.519527+00:00'}</t>
+          <t>{'status': 'ok', 'inception': '2000-01-03', 'rows': 6728, 'fetched_utc': '2026-10-04T19:22:06.865102+00:00'}</t>
         </is>
       </c>
     </row>
@@ -5630,7 +5630,7 @@
       </c>
       <c r="D13" s="17" t="inlineStr">
         <is>
-          <t>{'status': 'ok', 'inception': '2003-09-29', 'rows': 5790, 'fetched_utc': '2026-10-04T18:51:43.521581+00:00'}</t>
+          <t>{'status': 'ok', 'inception': '2003-09-29', 'rows': 5790, 'fetched_utc': '2026-10-04T19:22:06.866804+00:00'}</t>
         </is>
       </c>
     </row>

</xml_diff>